<commit_message>
Color coded board layout
</commit_message>
<xml_diff>
--- a/data/ClueLayout.xlsx
+++ b/data/ClueLayout.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10209"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/340AA63496B75636/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/chloemillham/eclipse-workspace/ClueGame/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="349" documentId="11_0B1D56BE9CDCCE836B02CE7A5FB0D4A9BBFD1C62" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0D935BFC-3205-4580-A9FB-6ADE1D4BBD8E}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8BF5EC0-9015-9B4C-8716-FE3A69525C9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
@@ -36,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="840" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="848" uniqueCount="45">
   <si>
     <t>GO</t>
   </si>
@@ -147,6 +146,30 @@
   </si>
   <si>
     <t>W*</t>
+  </si>
+  <si>
+    <t>Light yellow: Door Direction Tests (in FileInitTests)</t>
+  </si>
+  <si>
+    <t>Gray: room tests (in FileInitTests)</t>
+  </si>
+  <si>
+    <t>Yellow: adjacency from rooms and doors</t>
+  </si>
+  <si>
+    <t>Orange: adjacency walkways</t>
+  </si>
+  <si>
+    <t>Pink: walkway tests</t>
+  </si>
+  <si>
+    <t>Blue: target tests</t>
+  </si>
+  <si>
+    <t>Number of doors: 13</t>
+  </si>
+  <si>
+    <t>Red: player block tests</t>
   </si>
 </sst>
 </file>
@@ -162,7 +185,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="16">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -205,6 +228,54 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF59FF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -218,7 +289,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -241,6 +312,31 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -249,12 +345,15 @@
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleMedium9"/>
   <colors>
     <mruColors>
+      <color rgb="FFFF0000"/>
+      <color rgb="FFFF59FF"/>
+      <color rgb="FFFFFF7D"/>
       <color rgb="FFDDF7D2"/>
       <color rgb="FFFCFCD9"/>
+      <color rgb="FFFFFC00"/>
       <color rgb="FF87353D"/>
       <color rgb="FF6B131C"/>
       <color rgb="FF8C5687"/>
-      <color rgb="FFFFFF7D"/>
     </mruColors>
   </colors>
   <extLst>
@@ -585,19 +684,21 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AC31"/>
-  <sheetFormatPr defaultColWidth="3.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:AF31"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="3.5" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="3.5703125" style="1"/>
-    <col min="2" max="2" width="3.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="13" width="3.5703125" style="1"/>
-    <col min="14" max="15" width="3.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="16" max="28" width="3.5703125" style="1"/>
-    <col min="29" max="29" width="3.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="30" max="16384" width="3.5703125" style="1"/>
+    <col min="1" max="1" width="3.5" style="1"/>
+    <col min="2" max="2" width="3.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="13" width="3.5" style="1"/>
+    <col min="14" max="15" width="3.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="16" max="28" width="3.5" style="1"/>
+    <col min="29" max="29" width="3.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="30" max="31" width="3.5" style="1"/>
+    <col min="32" max="32" width="37.83203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="33" max="16384" width="3.5" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:32" x14ac:dyDescent="0.2">
       <c r="B1" s="1">
         <v>0</v>
       </c>
@@ -682,8 +783,11 @@
       <c r="AC1" s="1">
         <v>27</v>
       </c>
+      <c r="AF1" s="8" t="s">
+        <v>43</v>
+      </c>
     </row>
-    <row r="2" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A2" s="1">
         <v>0</v>
       </c>
@@ -771,8 +875,11 @@
       <c r="AC2" s="4" t="s">
         <v>3</v>
       </c>
+      <c r="AF2" s="9" t="s">
+        <v>37</v>
+      </c>
     </row>
-    <row r="3" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A3" s="1">
         <v>1</v>
       </c>
@@ -860,8 +967,11 @@
       <c r="AC3" s="5" t="s">
         <v>6</v>
       </c>
+      <c r="AF3" s="10" t="s">
+        <v>38</v>
+      </c>
     </row>
-    <row r="4" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A4" s="1">
         <v>2</v>
       </c>
@@ -949,8 +1059,9 @@
       <c r="AC4" s="2" t="s">
         <v>9</v>
       </c>
+      <c r="AF4"/>
     </row>
-    <row r="5" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A5" s="1">
         <v>3</v>
       </c>
@@ -963,7 +1074,7 @@
       <c r="D5" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="E5" s="7" t="s">
+      <c r="E5" s="18" t="s">
         <v>10</v>
       </c>
       <c r="F5" s="2" t="s">
@@ -1014,7 +1125,7 @@
       <c r="U5" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="V5" s="3" t="s">
+      <c r="V5" s="18" t="s">
         <v>2</v>
       </c>
       <c r="W5" s="3" t="s">
@@ -1038,8 +1149,11 @@
       <c r="AC5" s="2" t="s">
         <v>9</v>
       </c>
+      <c r="AF5" s="14" t="s">
+        <v>39</v>
+      </c>
     </row>
-    <row r="6" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A6" s="1">
         <v>4</v>
       </c>
@@ -1097,10 +1211,10 @@
       <c r="S6" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="T6" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="U6" s="3" t="s">
+      <c r="T6" s="18" t="s">
+        <v>2</v>
+      </c>
+      <c r="U6" s="15" t="s">
         <v>2</v>
       </c>
       <c r="V6" s="2" t="s">
@@ -1127,8 +1241,11 @@
       <c r="AC6" s="2" t="s">
         <v>9</v>
       </c>
+      <c r="AF6" s="11" t="s">
+        <v>40</v>
+      </c>
     </row>
-    <row r="7" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A7" s="1">
         <v>5</v>
       </c>
@@ -1180,7 +1297,7 @@
       <c r="Q7" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="R7" s="3" t="s">
+      <c r="R7" s="18" t="s">
         <v>2</v>
       </c>
       <c r="S7" s="3" t="s">
@@ -1189,7 +1306,7 @@
       <c r="T7" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="U7" s="6" t="s">
+      <c r="U7" s="18" t="s">
         <v>12</v>
       </c>
       <c r="V7" s="2" t="s">
@@ -1216,8 +1333,11 @@
       <c r="AC7" s="2" t="s">
         <v>9</v>
       </c>
+      <c r="AF7" s="17" t="s">
+        <v>41</v>
+      </c>
     </row>
-    <row r="8" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A8" s="1">
         <v>6</v>
       </c>
@@ -1239,10 +1359,10 @@
       <c r="G8" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="H8" s="6" t="s">
+      <c r="H8" s="13" t="s">
         <v>14</v>
       </c>
-      <c r="I8" s="3" t="s">
+      <c r="I8" s="18" t="s">
         <v>2</v>
       </c>
       <c r="J8" s="3" t="s">
@@ -1305,8 +1425,11 @@
       <c r="AC8" s="2" t="s">
         <v>9</v>
       </c>
+      <c r="AF8" s="12" t="s">
+        <v>42</v>
+      </c>
     </row>
-    <row r="9" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A9" s="1">
         <v>7</v>
       </c>
@@ -1328,10 +1451,10 @@
       <c r="G9" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="H9" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="I9" s="3" t="s">
+      <c r="H9" s="18" t="s">
+        <v>2</v>
+      </c>
+      <c r="I9" s="18" t="s">
         <v>2</v>
       </c>
       <c r="J9" s="3" t="s">
@@ -1367,7 +1490,7 @@
       <c r="T9" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="U9" s="3" t="s">
+      <c r="U9" s="18" t="s">
         <v>2</v>
       </c>
       <c r="V9" s="2" t="s">
@@ -1394,8 +1517,11 @@
       <c r="AC9" s="2" t="s">
         <v>9</v>
       </c>
+      <c r="AF9" s="19" t="s">
+        <v>44</v>
+      </c>
     </row>
-    <row r="10" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A10" s="1">
         <v>8</v>
       </c>
@@ -1417,13 +1543,13 @@
       <c r="G10" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="H10" s="3" t="s">
+      <c r="H10" s="18" t="s">
         <v>2</v>
       </c>
       <c r="I10" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="J10" s="3" t="s">
+      <c r="J10" s="15" t="s">
         <v>2</v>
       </c>
       <c r="K10" s="3" t="s">
@@ -1484,7 +1610,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="11" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A11" s="1">
         <v>9</v>
       </c>
@@ -1573,7 +1699,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="12" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A12" s="1">
         <v>10</v>
       </c>
@@ -1662,7 +1788,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="13" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A13" s="1">
         <v>11</v>
       </c>
@@ -1751,7 +1877,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="14" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A14" s="1">
         <v>12</v>
       </c>
@@ -1840,7 +1966,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="15" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A15" s="1">
         <v>13</v>
       </c>
@@ -1874,7 +2000,7 @@
       <c r="K15" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="L15" s="3" t="s">
+      <c r="L15" s="18" t="s">
         <v>2</v>
       </c>
       <c r="M15" s="3" t="s">
@@ -1901,7 +2027,7 @@
       <c r="T15" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="U15" s="6" t="s">
+      <c r="U15" s="20" t="s">
         <v>12</v>
       </c>
       <c r="V15" s="2" t="s">
@@ -1916,7 +2042,7 @@
       <c r="Y15" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="Z15" s="7" t="s">
+      <c r="Z15" s="20" t="s">
         <v>20</v>
       </c>
       <c r="AA15" s="2" t="s">
@@ -1929,7 +2055,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="16" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A16" s="1">
         <v>14</v>
       </c>
@@ -1942,7 +2068,7 @@
       <c r="D16" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="E16" s="7" t="s">
+      <c r="E16" s="20" t="s">
         <v>21</v>
       </c>
       <c r="F16" s="2" t="s">
@@ -1969,16 +2095,16 @@
       <c r="M16" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="N16" s="6" t="s">
+      <c r="N16" s="18" t="s">
         <v>22</v>
       </c>
       <c r="O16" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="P16" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="Q16" s="3" t="s">
+      <c r="P16" s="18" t="s">
+        <v>2</v>
+      </c>
+      <c r="Q16" s="18" t="s">
         <v>2</v>
       </c>
       <c r="R16" s="3" t="s">
@@ -2005,7 +2131,7 @@
       <c r="Y16" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="Z16" s="2" t="s">
+      <c r="Z16" s="13" t="s">
         <v>17</v>
       </c>
       <c r="AA16" s="2" t="s">
@@ -2018,7 +2144,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="17" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A17" s="1">
         <v>15</v>
       </c>
@@ -2107,7 +2233,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="18" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A18" s="1">
         <v>16</v>
       </c>
@@ -2129,7 +2255,7 @@
       <c r="G18" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="H18" s="3" t="s">
+      <c r="H18" s="20" t="s">
         <v>2</v>
       </c>
       <c r="I18" s="3" t="s">
@@ -2138,7 +2264,7 @@
       <c r="J18" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="K18" s="3" t="s">
+      <c r="K18" s="20" t="s">
         <v>2</v>
       </c>
       <c r="L18" s="2" t="s">
@@ -2196,7 +2322,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="19" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A19" s="1">
         <v>17</v>
       </c>
@@ -2224,7 +2350,7 @@
       <c r="I19" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="J19" s="3" t="s">
+      <c r="J19" s="20" t="s">
         <v>2</v>
       </c>
       <c r="K19" s="3" t="s">
@@ -2266,7 +2392,7 @@
       <c r="W19" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="X19" s="6" t="s">
+      <c r="X19" s="13" t="s">
         <v>15</v>
       </c>
       <c r="Y19" s="2" t="s">
@@ -2285,7 +2411,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="20" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A20" s="1">
         <v>18</v>
       </c>
@@ -2301,22 +2427,22 @@
       <c r="E20" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="F20" s="3" t="s">
+      <c r="F20" s="20" t="s">
         <v>2</v>
       </c>
       <c r="G20" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="H20" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="I20" s="3" t="s">
+      <c r="H20" s="20" t="s">
+        <v>2</v>
+      </c>
+      <c r="I20" s="20" t="s">
         <v>2</v>
       </c>
       <c r="J20" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="K20" s="3" t="s">
+      <c r="K20" s="20" t="s">
         <v>2</v>
       </c>
       <c r="L20" s="2" t="s">
@@ -2370,11 +2496,11 @@
       <c r="AB20" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="AC20" s="3" t="s">
+      <c r="AC20" s="15" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="21" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A21" s="1">
         <v>19</v>
       </c>
@@ -2393,7 +2519,7 @@
       <c r="F21" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="G21" s="3" t="s">
+      <c r="G21" s="20" t="s">
         <v>2</v>
       </c>
       <c r="H21" s="3" t="s">
@@ -2402,7 +2528,7 @@
       <c r="I21" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="J21" s="3" t="s">
+      <c r="J21" s="20" t="s">
         <v>2</v>
       </c>
       <c r="K21" s="3" t="s">
@@ -2429,13 +2555,13 @@
       <c r="R21" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="S21" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="T21" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="U21" s="3" t="s">
+      <c r="S21" s="16" t="s">
+        <v>2</v>
+      </c>
+      <c r="T21" s="16" t="s">
+        <v>2</v>
+      </c>
+      <c r="U21" s="16" t="s">
         <v>2</v>
       </c>
       <c r="V21" s="3" t="s">
@@ -2463,7 +2589,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="22" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A22" s="1">
         <v>20</v>
       </c>
@@ -2500,16 +2626,16 @@
       <c r="L22" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="M22" s="3" t="s">
+      <c r="M22" s="18" t="s">
         <v>2</v>
       </c>
       <c r="N22" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="O22" s="6" t="s">
+      <c r="O22" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="P22" s="6" t="s">
+      <c r="P22" s="18" t="s">
         <v>15</v>
       </c>
       <c r="Q22" s="3" t="s">
@@ -2521,19 +2647,19 @@
       <c r="S22" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="T22" s="3" t="s">
+      <c r="T22" s="16" t="s">
         <v>2</v>
       </c>
       <c r="U22" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="V22" s="3" t="s">
+      <c r="V22" s="16" t="s">
         <v>2</v>
       </c>
       <c r="W22" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="X22" s="3" t="s">
+      <c r="X22" s="16" t="s">
         <v>2</v>
       </c>
       <c r="Y22" s="3" t="s">
@@ -2552,7 +2678,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="23" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A23" s="1">
         <v>21</v>
       </c>
@@ -2601,7 +2727,7 @@
       <c r="P23" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="Q23" s="3" t="s">
+      <c r="Q23" s="18" t="s">
         <v>2</v>
       </c>
       <c r="R23" s="3" t="s">
@@ -2613,7 +2739,7 @@
       <c r="T23" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="U23" s="3" t="s">
+      <c r="U23" s="16" t="s">
         <v>2</v>
       </c>
       <c r="V23" s="3" t="s">
@@ -2622,7 +2748,7 @@
       <c r="W23" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="X23" s="3" t="s">
+      <c r="X23" s="16" t="s">
         <v>2</v>
       </c>
       <c r="Y23" s="2" t="s">
@@ -2641,7 +2767,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="24" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A24" s="1">
         <v>22</v>
       </c>
@@ -2684,7 +2810,7 @@
       <c r="N24" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="O24" s="3" t="s">
+      <c r="O24" s="18" t="s">
         <v>2</v>
       </c>
       <c r="P24" s="3" t="s">
@@ -2730,7 +2856,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="25" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A25" s="1">
         <v>23</v>
       </c>
@@ -2743,7 +2869,7 @@
       <c r="D25" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="E25" s="7" t="s">
+      <c r="E25" s="13" t="s">
         <v>30</v>
       </c>
       <c r="F25" s="2" t="s">
@@ -2776,7 +2902,7 @@
       <c r="O25" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="P25" s="6" t="s">
+      <c r="P25" s="18" t="s">
         <v>22</v>
       </c>
       <c r="Q25" s="3" t="s">
@@ -2791,7 +2917,7 @@
       <c r="T25" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="U25" s="6" t="s">
+      <c r="U25" s="16" t="s">
         <v>12</v>
       </c>
       <c r="V25" s="2" t="s">
@@ -2819,7 +2945,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="26" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A26" s="1">
         <v>24</v>
       </c>
@@ -2895,7 +3021,7 @@
       <c r="Y26" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="Z26" s="7" t="s">
+      <c r="Z26" s="16" t="s">
         <v>33</v>
       </c>
       <c r="AA26" s="2" t="s">
@@ -2908,7 +3034,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="27" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A27" s="1">
         <v>25</v>
       </c>
@@ -2997,7 +3123,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="28" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A28" s="1">
         <v>26</v>
       </c>
@@ -3086,7 +3212,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="29" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A29" s="1">
         <v>27</v>
       </c>
@@ -3108,7 +3234,7 @@
       <c r="G29" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="H29" s="3" t="s">
+      <c r="H29" s="15" t="s">
         <v>2</v>
       </c>
       <c r="I29" s="3" t="s">
@@ -3175,7 +3301,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="30" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A30" s="1">
         <v>28</v>
       </c>
@@ -3264,7 +3390,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="31" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A31" s="1">
         <v>29</v>
       </c>

</xml_diff>